<commit_message>
221 F5b: out-of-run screens in English, 补充三 wording fixes
Base (home, warehouse, sell, tech, codex, achievements), settings and
slots screens go through UiText (137 keys). Tech and achievement
descriptions gain an English field (techs.xlsx gets an 英文说明 column),
background and cursor names are bilingual, warehouse tabs use digits in
English, and the Fight / Continue buttons switch to English art.
补充三: node type condition shows short names, loot bias shows tag
names, 满级 merged into 满阶, trig.own_only reworded, tech panel hint
says above.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018nu316eEhzvyxZFyrEBn2i
</commit_message>
<xml_diff>
--- a/docs/techs.xlsx
+++ b/docs/techs.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -441,6 +441,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -462,6 +463,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
@@ -544,101 +546,114 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>效果构件</t>
+          <t>英文说明</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>RunRegistry.TECH_EFFECTS 里的类型：warehouse_pages / tech_safe_size / tech_run_buff / tech_belt_grant</t>
+          <t>descriptions.en，可空；不写数字（TextLint）</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>构件参数（JSON）</t>
+          <t>效果构件</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>构件自己的字段：tech_safe_size 填 {"cols": 0, "rows": 1}；tech_run_buff 填 {"effect": "&lt;RUN_EFFECTS 里的类型&gt;"}，每级的 run_buff 由工具生成（id = tech_&lt;id&gt;_&lt;级&gt;，scope META）</t>
+          <t>RunRegistry.TECH_EFFECTS 里的类型：warehouse_pages / tech_safe_size / tech_run_buff / tech_belt_grant</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>构件参数（JSON）</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>构件自己的字段：tech_safe_size 填 {"cols": 0, "rows": 1}；tech_run_buff 填 {"effect": "&lt;RUN_EFFECTS 里的类型&gt;"}，每级的 run_buff 由工具生成（id = tech_&lt;id&gt;_&lt;级&gt;，scope META）</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>每级说明模板</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>只 tech_run_buff 用：生成的 run_buff 的 description，占位符照 docs/text-placeholders.md，不写数字</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
+    <row r="18"/>
+    <row r="19">
+      <c r="A19" t="inlineStr">
         <is>
           <t>等级表的列</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="1" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="1" t="inlineStr">
         <is>
           <t>科技 id</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>对应节点表的 id；一个科技有几行就有几级，级号从 1 起连续</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>级</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>升到第几级</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>钱</t>
+          <t>级</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>这一级要的钱（TechTier.funds），整数</t>
+          <t>升到第几级</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>材料</t>
+          <t>钱</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>道具 id: 数量，多个用「；」分开，如 steel_ingot: 2；rivet_box: 1。空 = 不要材料（TechTier.items）</t>
+          <t>这一级要的钱（TechTier.funds），整数</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t>材料</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>道具 id: 数量，多个用「；」分开，如 steel_ingot: 2；rivet_box: 1。空 = 不要材料（TechTier.items）</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
           <t>效果参数（JSON）</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>只 tech_run_buff 用：这一级 run_buff 效果的参数，如 {"amount": 3}；空 = 全用默认值。别的构件这格留空（它们按级数自己算）</t>
         </is>
@@ -655,7 +670,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:K12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -706,17 +721,22 @@
           <t>说明</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>英文说明</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>效果构件</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>构件参数（JSON）</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>每级说明模板</t>
         </is>
@@ -756,15 +776,20 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
+          <t>Set out with extra money: a percentage of the character's own starting money.</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
           <t>tech_run_buff</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>{"effect": "starting_funds_bonus"}</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>开局钱 {starting_funds_bonus_percent|signed}%</t>
         </is>
@@ -804,10 +829,15 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
+          <t>The safe in a run gets more cells, so more is kept even if you fail to extract.</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
           <t>tech_safe_size</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>{"rows": 1}</t>
         </is>
@@ -842,6 +872,11 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
+          <t>One more Warehouse page for what you bring back; each page is separate, switch with the tabs on the left.</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
           <t>warehouse_pages</t>
         </is>
       </c>
@@ -875,15 +910,20 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
+          <t>Higher max Vitality, so you travel further on the map: a percentage of the character's own max Vitality.</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
           <t>tech_run_buff</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>{"effect": "vitality_max_bonus"}</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>体力上限 {vitality_max_bonus_percent|signed}%</t>
         </is>
@@ -923,15 +963,20 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
+          <t>Lose less Vitality when you lose a battle, but always at least one point.</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
           <t>tech_run_buff</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>{"effect": "loss_discount"}</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>打输了少扣 {loss_discount_amount} 点体力（最少扣一点）</t>
         </is>
@@ -971,15 +1016,20 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
+          <t>Higher max Health at the start: a percentage of the character's own Health.</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
           <t>tech_run_buff</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>{"effect": "stat_bonus"}</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>开局生命 {stat_bonus_amount|signed}%</t>
         </is>
@@ -1019,15 +1069,20 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
+          <t>Enemies drop their things more often.</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
           <t>tech_run_buff</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>{"effect": "luck_bonus"}</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>幸运 {luck_bonus_amount|signed}：敌人的东西更容易掉</t>
         </is>
@@ -1067,15 +1122,20 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
+          <t>Carry more before it gets heavy: a percentage of the character's own Load limit.</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
           <t>tech_run_buff</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>{"effect": "carry_capacity_bonus"}</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>负重上限 {carry_capacity_bonus_percent|signed}%</t>
         </is>
@@ -1115,15 +1175,20 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
+          <t>Hidden hunters become visible once they come close enough.</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
           <t>tech_run_buff</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="J10" t="inlineStr">
         <is>
           <t>{"effect": "scout_range"}</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>侦察距离 {scout_range_range}</t>
         </is>
@@ -1158,15 +1223,20 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
+          <t>Search each search spot a few more times.</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
           <t>tech_run_buff</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="J11" t="inlineStr">
         <is>
           <t>{"effect": "extra_searches"}</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t>每个搜索点多搜 {extra_searches_amount} 次</t>
         </is>
@@ -1206,15 +1276,20 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
+          <t>Shop prices are lower.</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
           <t>tech_run_buff</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="J12" t="inlineStr">
         <is>
           <t>{"effect": "shop_price_mult"}</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t>商店售价 ×{shop_price_mult_factor}</t>
         </is>

</xml_diff>

<commit_message>
229 tech page full tree + battle replay tidy (v3.82)
- Tech page: tree on the left over the stretched hide paper, wax/parchment
  detail board on the right; hand-in zone removed (materials hand in from
  their ledger row); three column header tags (Logistics / Physique /
  Exploration); 3 requires re-chained so the tree reads left to right.
- Battle replay: HP / stamina bars show numbers only, the battle report
  line is gone, the continue button switches to win / lose flag art when
  it lands.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018nu316eEhzvyxZFyrEBn2i
</commit_message>
<xml_diff>
--- a/docs/techs.xlsx
+++ b/docs/techs.xlsx
@@ -441,7 +441,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -463,7 +462,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
@@ -591,7 +589,6 @@
         </is>
       </c>
     </row>
-    <row r="18"/>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
@@ -953,7 +950,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>endurance</t>
+          <t>sinew</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -1165,7 +1162,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>luck、bargain</t>
+          <t>bargain</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1266,7 +1263,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>thorough_search</t>
+          <t>luck</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">

</xml_diff>